<commit_message>
Resolve the five open decisions from data; model numbers fill documents automatically
- Critical illness sized by need at HK$1.5M each (model premium input
  HK$113.6K average); ESG base HK$10.47M; Carmen 60% equity; card and tax
  stated as case-based assumptions with recommendations that hold either way
- model: export_numbers() writes figures/numbers.json (59 values);
  document/fill.py fills {{key}} placeholders; render.py fills before printing
- manuscript, section 3 mock-up and template now use placeholders; drafts
  and outline point to the manuscript as the single source

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/wong_model.xlsx
+++ b/model/wong_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\finplan\finplan\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECFA40C-1A85-43A1-8458-488055C4C821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8E23D6-C4E4-4BE9-9ED1-5271BC2B6A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -235,7 +235,7 @@
     <t>Insurance premiums (Lookbua, TBC)</t>
   </si>
   <si>
-    <t>parents' new cover, avg a year to 2036: DI 37K, term life 7K, CI 2.75M each ~96K avg (Bowtie Aug 2026), VHIS 15K. Paid until Adrian retires</t>
+    <t>parents' new cover, avg a year to 2036: DI 37K, term life 7K, CI 1.5M each ~55K avg (needs-based, Bowtie Aug 2026), VHIS 15K. Paid until Adrian retires</t>
   </si>
   <si>
     <t>MEDICAL (methodology §1)</t>
@@ -1693,7 +1693,7 @@
         <v>64</v>
       </c>
       <c r="B42" s="8">
-        <v>159000</v>
+        <v>113600</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>65</v>
@@ -5797,7 +5797,7 @@
       </c>
       <c r="Q4" s="16">
         <f>D4+E4-H4-I4+J4-K4-L4-M4-N4+O4+P4-IF($A4&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>631230</v>
+        <v>676630</v>
       </c>
       <c r="R4" s="16">
         <f>BalanceSheet!$B$37</f>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="U4" s="16">
         <f t="shared" ref="U4:U50" si="2">MAX(R4+S4+Q4+T4,0)</f>
-        <v>10891150</v>
+        <v>10936550</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -5882,15 +5882,15 @@
       </c>
       <c r="Q5" s="16">
         <f>D5+E5-H5-I5+J5-K5-L5-M5-N5+O5+P5-IF($A5&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>656733.00000000012</v>
+        <v>702133.00000000012</v>
       </c>
       <c r="R5" s="16">
         <f t="shared" ref="R5:R50" si="3">U4</f>
-        <v>10891150</v>
+        <v>10936550</v>
       </c>
       <c r="S5" s="16">
         <f>R5*Inputs!$B$35</f>
-        <v>522775.2</v>
+        <v>524954.4</v>
       </c>
       <c r="T5" s="16">
         <f>IF($A5=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="U5" s="16">
         <f t="shared" si="2"/>
-        <v>12070658.199999999</v>
+        <v>12163637.4</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
@@ -5967,15 +5967,15 @@
       </c>
       <c r="Q6" s="16">
         <f>D6+E6-H6-I6+J6-K6-L6-M6-N6+O6+P6-IF($A6&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>21612.615000000107</v>
+        <v>67012.615000000107</v>
       </c>
       <c r="R6" s="16">
         <f t="shared" si="3"/>
-        <v>12070658.199999999</v>
+        <v>12163637.4</v>
       </c>
       <c r="S6" s="16">
         <f>R6*Inputs!$B$35</f>
-        <v>579391.59360000002</v>
+        <v>583854.59519999998</v>
       </c>
       <c r="T6" s="16">
         <f>IF($A6=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="U6" s="16">
         <f t="shared" si="2"/>
-        <v>12671662.408599999</v>
+        <v>12814504.610200001</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
@@ -6052,15 +6052,15 @@
       </c>
       <c r="Q7" s="16">
         <f>D7+E7-H7-I7+J7-K7-L7-M7-N7+O7+P7-IF($A7&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>15822.931574999937</v>
+        <v>61222.931574999937</v>
       </c>
       <c r="R7" s="16">
         <f t="shared" si="3"/>
-        <v>12671662.408599999</v>
+        <v>12814504.610200001</v>
       </c>
       <c r="S7" s="16">
         <f>R7*Inputs!$B$35</f>
-        <v>608239.79561279994</v>
+        <v>615096.22128960001</v>
       </c>
       <c r="T7" s="16">
         <f>IF($A7=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="U7" s="16">
         <f t="shared" si="2"/>
-        <v>13295725.1357878</v>
+        <v>13490823.763064601</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
@@ -6137,15 +6137,15 @@
       </c>
       <c r="Q8" s="16">
         <f>D8+E8-H8-I8+J8-K8-L8-M8-N8+O8+P8-IF($A8&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>9315.2286003751215</v>
+        <v>54715.228600375121</v>
       </c>
       <c r="R8" s="16">
         <f t="shared" si="3"/>
-        <v>13295725.1357878</v>
+        <v>13490823.763064601</v>
       </c>
       <c r="S8" s="16">
         <f>R8*Inputs!$B$35</f>
-        <v>638194.8065178144</v>
+        <v>647559.54062710085</v>
       </c>
       <c r="T8" s="16">
         <f>IF($A8=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6153,7 +6153,7 @@
       </c>
       <c r="U8" s="16">
         <f t="shared" si="2"/>
-        <v>13943235.170905991</v>
+        <v>14193098.532292077</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
@@ -6222,15 +6222,15 @@
       </c>
       <c r="Q9" s="16">
         <f>D9+E9-H9-I9+J9-K9-L9-M9-N9+O9+P9-IF($A9&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>2037.8197634640383</v>
+        <v>47437.819763464038</v>
       </c>
       <c r="R9" s="16">
         <f t="shared" si="3"/>
-        <v>13943235.170905991</v>
+        <v>14193098.532292077</v>
       </c>
       <c r="S9" s="16">
         <f>R9*Inputs!$B$35</f>
-        <v>669275.28820348752</v>
+        <v>681268.72955001972</v>
       </c>
       <c r="T9" s="16">
         <f>IF($A9=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6238,7 +6238,7 @@
       </c>
       <c r="U9" s="16">
         <f t="shared" si="2"/>
-        <v>14614548.278872943</v>
+        <v>14921805.081605561</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
@@ -6307,15 +6307,15 @@
       </c>
       <c r="Q10" s="16">
         <f>D10+E10-H10-I10+J10-K10-L10-M10-N10+O10+P10-IF($A10&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>797993.27201907407</v>
+        <v>843393.27201907407</v>
       </c>
       <c r="R10" s="16">
         <f t="shared" si="3"/>
-        <v>14614548.278872943</v>
+        <v>14921805.081605561</v>
       </c>
       <c r="S10" s="16">
         <f>R10*Inputs!$B$35</f>
-        <v>701498.31738590123</v>
+        <v>716246.64391706698</v>
       </c>
       <c r="T10" s="16">
         <f>IF($A10=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="U10" s="16">
         <f t="shared" si="2"/>
-        <v>16114039.868277917</v>
+        <v>16481444.997541701</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
@@ -6392,15 +6392,15 @@
       </c>
       <c r="Q11" s="16">
         <f>D11+E11-H11-I11+J11-K11-L11-M11-N11+O11+P11-IF($A11&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>829211.56251829374</v>
+        <v>874611.56251829374</v>
       </c>
       <c r="R11" s="16">
         <f t="shared" si="3"/>
-        <v>16114039.868277917</v>
+        <v>16481444.997541701</v>
       </c>
       <c r="S11" s="16">
         <f>R11*Inputs!$B$35</f>
-        <v>773473.91367734002</v>
+        <v>791109.35988200165</v>
       </c>
       <c r="T11" s="16">
         <f>IF($A11=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="U11" s="16">
         <f t="shared" si="2"/>
-        <v>17716725.344473552</v>
+        <v>18147165.919941999</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -6477,15 +6477,15 @@
       </c>
       <c r="Q12" s="16">
         <f>D12+E12-H12-I12+J12-K12-L12-M12-N12+O12+P12-IF($A12&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>861495.73654095572</v>
+        <v>906895.73654095572</v>
       </c>
       <c r="R12" s="16">
         <f t="shared" si="3"/>
-        <v>17716725.344473552</v>
+        <v>18147165.919941999</v>
       </c>
       <c r="S12" s="16">
         <f>R12*Inputs!$B$35</f>
-        <v>850402.81653473049</v>
+        <v>871063.96415721602</v>
       </c>
       <c r="T12" s="16">
         <f>IF($A12=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6493,7 +6493,7 @@
       </c>
       <c r="U12" s="16">
         <f t="shared" si="2"/>
-        <v>19428623.897549238</v>
+        <v>19925125.62064017</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -6562,15 +6562,15 @@
       </c>
       <c r="Q13" s="16">
         <f>D13+E13-H13-I13+J13-K13-L13-M13-N13+O13+P13-IF($A13&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>894881.00396297663</v>
+        <v>940281.00396297663</v>
       </c>
       <c r="R13" s="16">
         <f t="shared" si="3"/>
-        <v>19428623.897549238</v>
+        <v>19925125.62064017</v>
       </c>
       <c r="S13" s="16">
         <f>R13*Inputs!$B$35</f>
-        <v>932573.94708236342</v>
+        <v>956406.02979072812</v>
       </c>
       <c r="T13" s="16">
         <f>IF($A13=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="U13" s="16">
         <f t="shared" si="2"/>
-        <v>21256078.848594576</v>
+        <v>21821812.654393874</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -6647,15 +6647,15 @@
       </c>
       <c r="Q14" s="16">
         <f>D14+E14-H14-I14+J14-K14-L14-M14-N14+O14+P14-IF($A14&lt;Inputs!$B$81,Inputs!$B$42,0)</f>
-        <v>929403.71179080242</v>
+        <v>974803.71179080242</v>
       </c>
       <c r="R14" s="16">
         <f t="shared" si="3"/>
-        <v>21256078.848594576</v>
+        <v>21821812.654393874</v>
       </c>
       <c r="S14" s="16">
         <f>R14*Inputs!$B$35</f>
-        <v>1020291.7847325397</v>
+        <v>1047447.007410906</v>
       </c>
       <c r="T14" s="16">
         <f>IF($A14=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="U14" s="16">
         <f t="shared" si="2"/>
-        <v>23205774.345117919</v>
+        <v>23844063.373595584</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
@@ -6736,11 +6736,11 @@
       </c>
       <c r="R15" s="23">
         <f t="shared" si="3"/>
-        <v>23205774.345117919</v>
+        <v>23844063.373595584</v>
       </c>
       <c r="S15" s="23">
         <f>R15*Inputs!$B$35</f>
-        <v>1113877.1685656602</v>
+        <v>1144515.041932588</v>
       </c>
       <c r="T15" s="23">
         <f>IF($A15=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="U15" s="23">
         <f t="shared" si="2"/>
-        <v>20348200.017858323</v>
+        <v>21017126.919702914</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -6821,11 +6821,11 @@
       </c>
       <c r="R16" s="16">
         <f t="shared" si="3"/>
-        <v>20348200.017858323</v>
+        <v>21017126.919702914</v>
       </c>
       <c r="S16" s="16">
         <f>R16*Inputs!$B$35</f>
-        <v>976713.60085719952</v>
+        <v>1008822.0921457398</v>
       </c>
       <c r="T16" s="16">
         <f>IF($A16=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="U16" s="16">
         <f t="shared" si="2"/>
-        <v>21473501.551300358</v>
+        <v>22174536.944433492</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -6906,11 +6906,11 @@
       </c>
       <c r="R17" s="23">
         <f t="shared" si="3"/>
-        <v>21473501.551300358</v>
+        <v>22174536.944433492</v>
       </c>
       <c r="S17" s="23">
         <f>R17*Inputs!$B$35</f>
-        <v>1030728.0744624172</v>
+        <v>1064377.7733328077</v>
       </c>
       <c r="T17" s="23">
         <f>IF($A17=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="U17" s="23">
         <f t="shared" si="2"/>
-        <v>21627347.557279609</v>
+        <v>22362032.649283133</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -6991,11 +6991,11 @@
       </c>
       <c r="R18" s="16">
         <f t="shared" si="3"/>
-        <v>21627347.557279609</v>
+        <v>22362032.649283133</v>
       </c>
       <c r="S18" s="16">
         <f>R18*Inputs!$B$35</f>
-        <v>1038112.6827494212</v>
+        <v>1073377.5671655904</v>
       </c>
       <c r="T18" s="16">
         <f>IF($A18=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="U18" s="16">
         <f t="shared" si="2"/>
-        <v>21744338.72678344</v>
+        <v>22514288.703203134</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -7076,11 +7076,11 @@
       </c>
       <c r="R19" s="16">
         <f t="shared" si="3"/>
-        <v>21744338.72678344</v>
+        <v>22514288.703203134</v>
       </c>
       <c r="S19" s="16">
         <f>R19*Inputs!$B$35</f>
-        <v>1043728.2588856051</v>
+        <v>1080685.8577537504</v>
       </c>
       <c r="T19" s="16">
         <f>IF($A19=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7088,7 +7088,7 @@
       </c>
       <c r="U19" s="16">
         <f t="shared" si="2"/>
-        <v>21819667.345723789</v>
+        <v>22626574.92101163</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -7161,11 +7161,11 @@
       </c>
       <c r="R20" s="16">
         <f t="shared" si="3"/>
-        <v>21819667.345723789</v>
+        <v>22626574.92101163</v>
       </c>
       <c r="S20" s="16">
         <f>R20*Inputs!$B$35</f>
-        <v>1047344.0325947419</v>
+        <v>1086075.5962085582</v>
       </c>
       <c r="T20" s="16">
         <f>IF($A20=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7173,7 +7173,7 @@
       </c>
       <c r="U20" s="16">
         <f t="shared" si="2"/>
-        <v>21847978.719372328</v>
+        <v>22693617.858273987</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -7246,11 +7246,11 @@
       </c>
       <c r="R21" s="16">
         <f t="shared" si="3"/>
-        <v>21847978.719372328</v>
+        <v>22693617.858273987</v>
       </c>
       <c r="S21" s="16">
         <f>R21*Inputs!$B$35</f>
-        <v>1048702.9785298717</v>
+        <v>1089293.6571971513</v>
       </c>
       <c r="T21" s="16">
         <f>IF($A21=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="U21" s="16">
         <f t="shared" si="2"/>
-        <v>21825201.059069425</v>
+        <v>22711430.876638364</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -7331,11 +7331,11 @@
       </c>
       <c r="R22" s="16">
         <f t="shared" si="3"/>
-        <v>21825201.059069425</v>
+        <v>22711430.876638364</v>
       </c>
       <c r="S22" s="16">
         <f>R22*Inputs!$B$35</f>
-        <v>1047609.6508353325</v>
+        <v>1090148.6820786416</v>
       </c>
       <c r="T22" s="16">
         <f>IF($A22=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="U22" s="16">
         <f t="shared" si="2"/>
-        <v>21745242.013943352</v>
+        <v>22674010.8627556</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -7416,11 +7416,11 @@
       </c>
       <c r="R23" s="16">
         <f t="shared" si="3"/>
-        <v>21745242.013943352</v>
+        <v>22674010.8627556</v>
       </c>
       <c r="S23" s="16">
         <f>R23*Inputs!$B$35</f>
-        <v>1043771.6166692809</v>
+        <v>1088352.5214122687</v>
       </c>
       <c r="T23" s="16">
         <f>IF($A23=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7428,7 +7428,7 @@
       </c>
       <c r="U23" s="16">
         <f t="shared" si="2"/>
-        <v>21601358.207723934</v>
+        <v>22574707.961279169</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -7501,11 +7501,11 @@
       </c>
       <c r="R24" s="16">
         <f t="shared" si="3"/>
-        <v>21601358.207723934</v>
+        <v>22574707.961279169</v>
       </c>
       <c r="S24" s="16">
         <f>R24*Inputs!$B$35</f>
-        <v>1036865.1939707488</v>
+        <v>1083585.9821414002</v>
       </c>
       <c r="T24" s="16">
         <f>IF($A24=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7513,7 +7513,7 @@
       </c>
       <c r="U24" s="16">
         <f t="shared" si="2"/>
-        <v>21386084.272740219</v>
+        <v>22406154.814466108</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -7586,11 +7586,11 @@
       </c>
       <c r="R25" s="16">
         <f t="shared" si="3"/>
-        <v>21386084.272740219</v>
+        <v>22406154.814466108</v>
       </c>
       <c r="S25" s="16">
         <f>R25*Inputs!$B$35</f>
-        <v>1026532.0450915305</v>
+        <v>1075495.4310943731</v>
       </c>
       <c r="T25" s="16">
         <f>IF($A25=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="U25" s="16">
         <f t="shared" si="2"/>
-        <v>21091153.949926905</v>
+        <v>22160187.87765564</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -7671,11 +7671,11 @@
       </c>
       <c r="R26" s="16">
         <f t="shared" si="3"/>
-        <v>21091153.949926905</v>
+        <v>22160187.87765564</v>
       </c>
       <c r="S26" s="16">
         <f>R26*Inputs!$B$35</f>
-        <v>1012375.3895964915</v>
+        <v>1063689.0181274707</v>
       </c>
       <c r="T26" s="16">
         <f>IF($A26=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7683,7 +7683,7 @@
       </c>
       <c r="U26" s="16">
         <f t="shared" si="2"/>
-        <v>20711268.788185466</v>
+        <v>21831616.34444518</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -7756,11 +7756,11 @@
       </c>
       <c r="R27" s="16">
         <f t="shared" si="3"/>
-        <v>20711268.788185466</v>
+        <v>21831616.34444518</v>
       </c>
       <c r="S27" s="16">
         <f>R27*Inputs!$B$35</f>
-        <v>994140.90183290234</v>
+        <v>1047917.5845333687</v>
       </c>
       <c r="T27" s="16">
         <f>IF($A27=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="U27" s="16">
         <f t="shared" si="2"/>
-        <v>20237279.403837793</v>
+        <v>21411403.642797973</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -7841,11 +7841,11 @@
       </c>
       <c r="R28" s="16">
         <f t="shared" si="3"/>
-        <v>20237279.403837793</v>
+        <v>21411403.642797973</v>
       </c>
       <c r="S28" s="16">
         <f>R28*Inputs!$B$35</f>
-        <v>971389.41138421407</v>
+        <v>1027747.3748543027</v>
       </c>
       <c r="T28" s="16">
         <f>IF($A28=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="U28" s="16">
         <f t="shared" si="2"/>
-        <v>19659116.101737805</v>
+        <v>20889598.304168075</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -7926,11 +7926,11 @@
       </c>
       <c r="R29" s="16">
         <f t="shared" si="3"/>
-        <v>19659116.101737805</v>
+        <v>20889598.304168075</v>
       </c>
       <c r="S29" s="16">
         <f>R29*Inputs!$B$35</f>
-        <v>943637.57288341469</v>
+        <v>1002700.7186000677</v>
       </c>
       <c r="T29" s="16">
         <f>IF($A29=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -7938,7 +7938,7 @@
       </c>
       <c r="U29" s="16">
         <f t="shared" si="2"/>
-        <v>18965694.279604044</v>
+        <v>20255239.627750967</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -8011,11 +8011,11 @@
       </c>
       <c r="R30" s="16">
         <f t="shared" si="3"/>
-        <v>18965694.279604044</v>
+        <v>20255239.627750967</v>
       </c>
       <c r="S30" s="16">
         <f>R30*Inputs!$B$35</f>
-        <v>910353.32542099408</v>
+        <v>972251.50213204639</v>
       </c>
       <c r="T30" s="16">
         <f>IF($A30=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8023,7 +8023,7 @@
       </c>
       <c r="U30" s="16">
         <f t="shared" si="2"/>
-        <v>18144809.834026922</v>
+        <v>19496253.358884897</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -8096,11 +8096,11 @@
       </c>
       <c r="R31" s="16">
         <f t="shared" si="3"/>
-        <v>18144809.834026922</v>
+        <v>19496253.358884897</v>
       </c>
       <c r="S31" s="16">
         <f>R31*Inputs!$B$35</f>
-        <v>870950.87203329219</v>
+        <v>935820.16122647503</v>
       </c>
       <c r="T31" s="16">
         <f>IF($A31=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="U31" s="16">
         <f t="shared" si="2"/>
-        <v>17189240.614425432</v>
+        <v>18605553.428476591</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -8181,11 +8181,11 @@
       </c>
       <c r="R32" s="16">
         <f t="shared" si="3"/>
-        <v>17189240.614425432</v>
+        <v>18605553.428476591</v>
       </c>
       <c r="S32" s="16">
         <f>R32*Inputs!$B$35</f>
-        <v>825083.54949242075</v>
+        <v>893066.56456687639</v>
       </c>
       <c r="T32" s="16">
         <f>IF($A32=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8193,7 +8193,7 @@
       </c>
       <c r="U32" s="16">
         <f t="shared" si="2"/>
-        <v>16085803.202489708</v>
+        <v>17570099.031615321</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -8266,11 +8266,11 @@
       </c>
       <c r="R33" s="16">
         <f t="shared" si="3"/>
-        <v>16085803.202489708</v>
+        <v>17570099.031615321</v>
       </c>
       <c r="S33" s="16">
         <f>R33*Inputs!$B$35</f>
-        <v>772118.55371950602</v>
+        <v>843364.7535175354</v>
       </c>
       <c r="T33" s="16">
         <f>IF($A33=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8278,7 +8278,7 @@
       </c>
       <c r="U33" s="16">
         <f t="shared" si="2"/>
-        <v>14820098.298671564</v>
+        <v>16375640.327595206</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -8351,11 +8351,11 @@
       </c>
       <c r="R34" s="23">
         <f t="shared" si="3"/>
-        <v>14820098.298671564</v>
+        <v>16375640.327595206</v>
       </c>
       <c r="S34" s="23">
         <f>R34*Inputs!$B$35</f>
-        <v>711364.71833623503</v>
+        <v>786030.73572456988</v>
       </c>
       <c r="T34" s="23">
         <f>IF($A34=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8363,7 +8363,7 @@
       </c>
       <c r="U34" s="23">
         <f t="shared" si="2"/>
-        <v>13376398.045838624</v>
+        <v>15006606.092150601</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -8436,11 +8436,11 @@
       </c>
       <c r="R35" s="16">
         <f t="shared" si="3"/>
-        <v>13376398.045838624</v>
+        <v>15006606.092150601</v>
       </c>
       <c r="S35" s="16">
         <f>R35*Inputs!$B$35</f>
-        <v>642067.10620025394</v>
+        <v>720317.0924232289</v>
       </c>
       <c r="T35" s="16">
         <f>IF($A35=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8448,7 +8448,7 @@
       </c>
       <c r="U35" s="16">
         <f t="shared" si="2"/>
-        <v>12288823.083724447</v>
+        <v>13997281.1162594</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -8521,11 +8521,11 @@
       </c>
       <c r="R36" s="16">
         <f t="shared" si="3"/>
-        <v>12288823.083724447</v>
+        <v>13997281.1162594</v>
       </c>
       <c r="S36" s="16">
         <f>R36*Inputs!$B$35</f>
-        <v>589863.5080187734</v>
+        <v>671869.49358045124</v>
       </c>
       <c r="T36" s="16">
         <f>IF($A36=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8533,7 +8533,7 @@
       </c>
       <c r="U36" s="16">
         <f t="shared" si="2"/>
-        <v>11066624.516588137</v>
+        <v>12857088.534684768</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -8606,11 +8606,11 @@
       </c>
       <c r="R37" s="16">
         <f t="shared" si="3"/>
-        <v>11066624.516588137</v>
+        <v>12857088.534684768</v>
       </c>
       <c r="S37" s="16">
         <f>R37*Inputs!$B$35</f>
-        <v>531197.97679623053</v>
+        <v>617140.24966486893</v>
       </c>
       <c r="T37" s="16">
         <f>IF($A37=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8618,7 +8618,7 @@
       </c>
       <c r="U37" s="16">
         <f t="shared" si="2"/>
-        <v>9698176.6432708651</v>
+        <v>11574582.934236135</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -8691,11 +8691,11 @@
       </c>
       <c r="R38" s="16">
         <f t="shared" si="3"/>
-        <v>9698176.6432708651</v>
+        <v>11574582.934236135</v>
       </c>
       <c r="S38" s="16">
         <f>R38*Inputs!$B$35</f>
-        <v>465512.47887700156</v>
+        <v>555579.98084333446</v>
       </c>
       <c r="T38" s="16">
         <f>IF($A38=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8703,7 +8703,7 @@
       </c>
       <c r="U38" s="16">
         <f t="shared" si="2"/>
-        <v>8170870.1266960986</v>
+        <v>10137343.919627702</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -8776,11 +8776,11 @@
       </c>
       <c r="R39" s="16">
         <f t="shared" si="3"/>
-        <v>8170870.1266960986</v>
+        <v>10137343.919627702</v>
       </c>
       <c r="S39" s="16">
         <f>R39*Inputs!$B$35</f>
-        <v>392201.76608141273</v>
+        <v>486592.50814212969</v>
       </c>
       <c r="T39" s="16">
         <f>IF($A39=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="U39" s="16">
         <f t="shared" si="2"/>
-        <v>6471025.8088223208</v>
+        <v>8531890.3438146412</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -8861,11 +8861,11 @@
       </c>
       <c r="R40" s="16">
         <f t="shared" si="3"/>
-        <v>6471025.8088223208</v>
+        <v>8531890.3438146412</v>
       </c>
       <c r="S40" s="16">
         <f>R40*Inputs!$B$35</f>
-        <v>310609.23882347142</v>
+        <v>409530.73650310282</v>
       </c>
       <c r="T40" s="16">
         <f>IF($A40=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8873,7 +8873,7 @@
       </c>
       <c r="U40" s="16">
         <f t="shared" si="2"/>
-        <v>4583800.7075582501</v>
+        <v>6743586.7402302008</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -8946,11 +8946,11 @@
       </c>
       <c r="R41" s="16">
         <f t="shared" si="3"/>
-        <v>4583800.7075582501</v>
+        <v>6743586.7402302008</v>
       </c>
       <c r="S41" s="16">
         <f>R41*Inputs!$B$35</f>
-        <v>220022.433962796</v>
+        <v>323692.16353104962</v>
       </c>
       <c r="T41" s="16">
         <f>IF($A41=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="U41" s="16">
         <f t="shared" si="2"/>
-        <v>2493085.4697103309</v>
+        <v>4756541.2319505364</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -9031,11 +9031,11 @@
       </c>
       <c r="R42" s="16">
         <f t="shared" si="3"/>
-        <v>2493085.4697103309</v>
+        <v>4756541.2319505364</v>
       </c>
       <c r="S42" s="16">
         <f>R42*Inputs!$B$35</f>
-        <v>119668.10254609589</v>
+        <v>228313.97913362575</v>
       </c>
       <c r="T42" s="16">
         <f>IF($A42=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -9043,7 +9043,7 @@
       </c>
       <c r="U42" s="16">
         <f t="shared" si="2"/>
-        <v>181392.485709175</v>
+        <v>2553494.1245369101</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -9116,11 +9116,11 @@
       </c>
       <c r="R43" s="16">
         <f t="shared" si="3"/>
-        <v>181392.485709175</v>
+        <v>2553494.1245369101</v>
       </c>
       <c r="S43" s="16">
         <f>R43*Inputs!$B$35</f>
-        <v>8706.8393140404005</v>
+        <v>122567.71797777168</v>
       </c>
       <c r="T43" s="16">
         <f>IF($A43=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="U43" s="16">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>115696.31455235416</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -9201,11 +9201,11 @@
       </c>
       <c r="R44" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>115696.31455235416</v>
       </c>
       <c r="S44" s="23">
         <f>R44*Inputs!$B$35</f>
-        <v>0</v>
+        <v>5553.4230985129998</v>
       </c>
       <c r="T44" s="23">
         <f>IF($A44=Inputs!$B$81,-Inputs!$B$38,0)</f>
@@ -9780,7 +9780,7 @@
       </c>
       <c r="B7" s="24">
         <f>Tax!B27-Inputs!$B$42</f>
-        <v>559230</v>
+        <v>604630</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="B14" s="24">
         <f>INDEX(Projection!U:U,MATCH(Inputs!$B$81,Projection!A:A,0))</f>
-        <v>20348200.017858323</v>
+        <v>21017126.919702914</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="B17" s="24">
         <f>INDEX(Projection!U:U,MATCH(Inputs!$B$81,Projection!A:A,0))/(1+Inputs!$B$5)^(Inputs!$B$81-Inputs!$B$80)</f>
-        <v>15508274.470191544</v>
+        <v>16018093.618086508</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="B19" s="26">
         <f>IFERROR(INDEX(Projection!A4:A50,MATCH(0,Projection!U4:U50,0)),0)</f>
-        <v>2065</v>
+        <v>2066</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B20" s="26">
         <f>IF(B19=0,"lasts",B19-1977)</f>
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>